<commit_message>
completed login and register pages with dataproviders except assertions
</commit_message>
<xml_diff>
--- a/july192025/Testng_sowmya/src/test/resources/testdata/TestNG_data.xlsx
+++ b/july192025/Testng_sowmya/src/test/resources/testdata/TestNG_data.xlsx
@@ -3,15 +3,19 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{764F6AA8-245A-4691-858A-901CF865306C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rahul\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5FEFEE-C367-442D-86D9-A58068853461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EB05B32A-5D5A-7149-A1FC-6A11C218CEA0}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{EB05B32A-5D5A-7149-A1FC-6A11C218CEA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
login page is done with all assertions
</commit_message>
<xml_diff>
--- a/july192025/Testng_sowmya/src/test/resources/testdata/TestNG_data.xlsx
+++ b/july192025/Testng_sowmya/src/test/resources/testdata/TestNG_data.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rahul\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5FEFEE-C367-442D-86D9-A58068853461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{33CDE666-92F8-418B-A5B0-0B7D11F43A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{EB05B32A-5D5A-7149-A1FC-6A11C218CEA0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EB05B32A-5D5A-7149-A1FC-6A11C218CEA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
all modules are working fine along with assertions
</commit_message>
<xml_diff>
--- a/july192025/Testng_sowmya/src/test/resources/testdata/TestNG_data.xlsx
+++ b/july192025/Testng_sowmya/src/test/resources/testdata/TestNG_data.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rahul\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5FEFEE-C367-442D-86D9-A58068853461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{181CC33E-6CF5-4490-83AF-8474B0308883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{EB05B32A-5D5A-7149-A1FC-6A11C218CEA0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EB05B32A-5D5A-7149-A1FC-6A11C218CEA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -163,9 +159,6 @@
     <t>Invalid Username and Password</t>
   </si>
   <si>
-    <t>missmathch password</t>
-  </si>
-  <si>
     <t>Login1</t>
   </si>
   <si>
@@ -227,6 +220,9 @@
   </si>
   <si>
     <t>Please fill out this field.</t>
+  </si>
+  <si>
+    <t>password_mismatch:The two password fields didn’t match.</t>
   </si>
 </sst>
 </file>
@@ -731,24 +727,24 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="21">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>4</v>
@@ -784,7 +780,7 @@
     </row>
     <row r="4" spans="1:9" ht="21">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="2"/>
@@ -802,7 +798,7 @@
     </row>
     <row r="5" spans="1:9" ht="21">
       <c r="A5" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="2"/>
@@ -886,44 +882,44 @@
     </row>
     <row r="10" spans="1:9" ht="34.950000000000003" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="H10" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I10" s="14"/>
     </row>
     <row r="11" spans="1:9" ht="21">
       <c r="A11" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>26</v>
       </c>
       <c r="C11" s="12"/>
       <c r="H11" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I11" s="14"/>
     </row>
     <row r="12" spans="1:9" ht="21">
       <c r="A12" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
         <v>27</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" ht="21">
       <c r="A13" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>26</v>
@@ -938,44 +934,44 @@
     </row>
     <row r="14" spans="1:9" ht="21">
       <c r="A14" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="H14" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I14" s="14"/>
     </row>
     <row r="15" spans="1:9" ht="21">
       <c r="A15" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="12"/>
       <c r="H15" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I15" s="14"/>
     </row>
     <row r="16" spans="1:9" ht="21">
       <c r="A16" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="12"/>
       <c r="C16" s="12" t="s">
         <v>5</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I16" s="14"/>
     </row>
     <row r="17" spans="1:9" ht="21">
       <c r="A17" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>26</v>
@@ -984,13 +980,13 @@
         <v>5</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I17" s="14"/>
     </row>
     <row r="18" spans="1:9" ht="21">
       <c r="A18" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>26</v>
@@ -999,15 +995,15 @@
         <v>5</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="21">
       <c r="A19" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>4</v>
@@ -1016,7 +1012,7 @@
         <v>5</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I19" s="15" t="s">
         <v>5</v>

</xml_diff>